<commit_message>
Latest files for 12/03/2026
</commit_message>
<xml_diff>
--- a/PhD Thesis Timeline.xlsx
+++ b/PhD Thesis Timeline.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ppit/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/ppit_student_unimelb_edu_au/Documents/Desktop/PhD-Thesis-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DD1AFA-1B1D-CF49-BA5A-312FDD1339BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{70DD1AFA-1B1D-CF49-BA5A-312FDD1339BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BAA9E1F-2BCF-DD43-8FE8-FC41276B5DCA}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18220" yWindow="-20200" windowWidth="29100" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Study 2 Timeline" sheetId="1" r:id="rId1"/>
@@ -64,9 +64,6 @@
     <t>XX</t>
   </si>
   <si>
-    <t>40 Semi-Structured Interviews</t>
-  </si>
-  <si>
     <t>Transcription &amp; Thematic Analysis</t>
   </si>
   <si>
@@ -260,6 +257,9 @@
   </si>
   <si>
     <t>Thesis Writeup &amp; Submission</t>
+  </si>
+  <si>
+    <t>20 Semi-Structured Interviews</t>
   </si>
 </sst>
 </file>
@@ -744,6 +744,30 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -769,30 +793,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1024,7 +1024,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1032,94 +1032,94 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="54">
+      <c r="D1" s="45">
         <v>2026</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="54"/>
-      <c r="O1" s="54"/>
-      <c r="P1" s="54">
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45">
         <v>2027</v>
       </c>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="54"/>
-      <c r="U1" s="54"/>
-      <c r="V1" s="54"/>
-      <c r="W1" s="54"/>
-      <c r="X1" s="54"/>
-      <c r="Y1" s="54"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="54"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="45"/>
+      <c r="U1" s="45"/>
+      <c r="V1" s="45"/>
+      <c r="W1" s="45"/>
+      <c r="X1" s="45"/>
+      <c r="Y1" s="45"/>
+      <c r="Z1" s="45"/>
+      <c r="AA1" s="45"/>
     </row>
     <row r="2" spans="1:27" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="56" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="56"/>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="56"/>
-      <c r="Q2" s="56"/>
-      <c r="R2" s="56"/>
-      <c r="S2" s="56"/>
-      <c r="T2" s="56"/>
-      <c r="U2" s="56"/>
-      <c r="V2" s="56"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="56"/>
-      <c r="Y2" s="56"/>
-      <c r="Z2" s="56"/>
-      <c r="AA2" s="56"/>
+      <c r="A2" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="47"/>
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+      <c r="U2" s="47"/>
+      <c r="V2" s="47"/>
+      <c r="W2" s="47"/>
+      <c r="X2" s="47"/>
+      <c r="Y2" s="47"/>
+      <c r="Z2" s="47"/>
+      <c r="AA2" s="47"/>
     </row>
     <row r="3" spans="1:27" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="56"/>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="56"/>
-      <c r="W3" s="56"/>
-      <c r="X3" s="56"/>
-      <c r="Y3" s="56"/>
-      <c r="Z3" s="56"/>
-      <c r="AA3" s="56"/>
+      <c r="A3" s="47"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="47"/>
+      <c r="P3" s="47"/>
+      <c r="Q3" s="47"/>
+      <c r="R3" s="47"/>
+      <c r="S3" s="47"/>
+      <c r="T3" s="47"/>
+      <c r="U3" s="47"/>
+      <c r="V3" s="47"/>
+      <c r="W3" s="47"/>
+      <c r="X3" s="47"/>
+      <c r="Y3" s="47"/>
+      <c r="Z3" s="47"/>
+      <c r="AA3" s="47"/>
     </row>
     <row r="4" spans="1:27" ht="20" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
@@ -1156,10 +1156,10 @@
         <v>11</v>
       </c>
       <c r="N4" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="O4" s="18" t="s">
         <v>27</v>
-      </c>
-      <c r="O4" s="18" t="s">
-        <v>28</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>2</v>
@@ -1192,18 +1192,18 @@
         <v>11</v>
       </c>
       <c r="Z4" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA4" s="18" t="s">
         <v>27</v>
-      </c>
-      <c r="AA4" s="18" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A5" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>12</v>
@@ -1238,17 +1238,17 @@
     <row r="6" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A6" s="6"/>
       <c r="B6" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>14</v>
+        <v>79</v>
       </c>
       <c r="D6" s="19"/>
-      <c r="E6" s="57" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
+      <c r="E6" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
       <c r="H6" s="19"/>
       <c r="I6" s="19"/>
       <c r="J6" s="19"/>
@@ -1273,17 +1273,17 @@
     <row r="7" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A7" s="6"/>
       <c r="B7" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7" s="19"/>
       <c r="E7" s="19"/>
-      <c r="F7" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="58"/>
+      <c r="F7" s="49" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="49"/>
       <c r="H7" s="19"/>
       <c r="I7" s="19"/>
       <c r="J7" s="19"/>
@@ -1332,13 +1332,13 @@
     </row>
     <row r="9" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A9" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" s="20"/>
       <c r="E9" s="20"/>
@@ -1370,10 +1370,10 @@
     <row r="10" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A10" s="6"/>
       <c r="B10" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D10" s="20"/>
       <c r="E10" s="20"/>
@@ -1405,10 +1405,10 @@
     <row r="11" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A11" s="6"/>
       <c r="B11" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D11" s="20"/>
       <c r="E11" s="20"/>
@@ -1463,23 +1463,23 @@
     </row>
     <row r="13" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A13" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D13" s="20"/>
       <c r="E13" s="20"/>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
       <c r="H13" s="20"/>
-      <c r="I13" s="59" t="s">
-        <v>13</v>
-      </c>
-      <c r="J13" s="59"/>
+      <c r="I13" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" s="50"/>
       <c r="K13" s="20"/>
       <c r="L13" s="20"/>
       <c r="M13" s="20"/>
@@ -1501,37 +1501,37 @@
     <row r="14" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A14" s="6"/>
       <c r="B14" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C14" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="55" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
-      <c r="J14" s="55"/>
-      <c r="K14" s="55"/>
-      <c r="L14" s="55"/>
-      <c r="M14" s="55"/>
-      <c r="N14" s="55"/>
-      <c r="O14" s="55"/>
-      <c r="P14" s="55"/>
-      <c r="Q14" s="55"/>
-      <c r="R14" s="55"/>
-      <c r="S14" s="55"/>
-      <c r="T14" s="55"/>
-      <c r="U14" s="55"/>
-      <c r="V14" s="55"/>
-      <c r="W14" s="55"/>
-      <c r="X14" s="55"/>
-      <c r="Y14" s="55"/>
-      <c r="Z14" s="55"/>
-      <c r="AA14" s="55"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46"/>
+      <c r="K14" s="46"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="46"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="46"/>
+      <c r="U14" s="46"/>
+      <c r="V14" s="46"/>
+      <c r="W14" s="46"/>
+      <c r="X14" s="46"/>
+      <c r="Y14" s="46"/>
+      <c r="Z14" s="46"/>
+      <c r="AA14" s="46"/>
     </row>
     <row r="15" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A15" s="10"/>
@@ -1560,13 +1560,13 @@
     </row>
     <row r="16" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A16" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
@@ -1574,10 +1574,10 @@
       <c r="G16" s="20"/>
       <c r="H16" s="20"/>
       <c r="I16" s="20"/>
-      <c r="J16" s="60" t="s">
-        <v>13</v>
-      </c>
-      <c r="K16" s="60"/>
+      <c r="J16" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" s="51"/>
       <c r="L16" s="20"/>
       <c r="M16" s="20"/>
       <c r="N16" s="20"/>
@@ -1598,10 +1598,10 @@
     <row r="17" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A17" s="6"/>
       <c r="B17" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D17" s="20"/>
       <c r="E17" s="20"/>
@@ -1656,13 +1656,13 @@
     </row>
     <row r="19" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A19" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" s="20"/>
       <c r="E19" s="20"/>
@@ -1672,10 +1672,10 @@
       <c r="I19" s="20"/>
       <c r="J19" s="20"/>
       <c r="K19" s="20"/>
-      <c r="L19" s="53" t="s">
-        <v>13</v>
-      </c>
-      <c r="M19" s="53"/>
+      <c r="L19" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="M19" s="44"/>
       <c r="N19" s="20"/>
       <c r="O19" s="20"/>
       <c r="P19" s="20"/>
@@ -1694,50 +1694,50 @@
     <row r="20" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A20" s="6"/>
       <c r="B20" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>73</v>
-      </c>
-      <c r="M20" s="49" t="s">
-        <v>13</v>
-      </c>
-      <c r="N20" s="49"/>
+        <v>72</v>
+      </c>
+      <c r="M20" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="N20" s="57"/>
     </row>
     <row r="21" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A21" s="6"/>
       <c r="B21" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="55" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="55"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="55"/>
-      <c r="K21" s="55"/>
-      <c r="L21" s="55"/>
-      <c r="M21" s="55"/>
-      <c r="N21" s="55"/>
-      <c r="O21" s="55"/>
-      <c r="P21" s="55"/>
-      <c r="Q21" s="55"/>
-      <c r="R21" s="55"/>
-      <c r="S21" s="55"/>
-      <c r="T21" s="55"/>
-      <c r="U21" s="55"/>
-      <c r="V21" s="55"/>
-      <c r="W21" s="55"/>
-      <c r="X21" s="55"/>
-      <c r="Y21" s="55"/>
-      <c r="Z21" s="55"/>
-      <c r="AA21" s="55"/>
+        <v>17</v>
+      </c>
+      <c r="D21" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46"/>
+      <c r="K21" s="46"/>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="46"/>
+      <c r="O21" s="46"/>
+      <c r="P21" s="46"/>
+      <c r="Q21" s="46"/>
+      <c r="R21" s="46"/>
+      <c r="S21" s="46"/>
+      <c r="T21" s="46"/>
+      <c r="U21" s="46"/>
+      <c r="V21" s="46"/>
+      <c r="W21" s="46"/>
+      <c r="X21" s="46"/>
+      <c r="Y21" s="46"/>
+      <c r="Z21" s="46"/>
+      <c r="AA21" s="46"/>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A22" s="43"/>
@@ -1769,64 +1769,64 @@
       <c r="AA22" s="43"/>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A23" s="56" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="56"/>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
-      <c r="J23" s="56"/>
-      <c r="K23" s="56"/>
-      <c r="L23" s="56"/>
-      <c r="M23" s="56"/>
-      <c r="N23" s="56"/>
-      <c r="O23" s="56"/>
-      <c r="P23" s="56"/>
-      <c r="Q23" s="56"/>
-      <c r="R23" s="56"/>
-      <c r="S23" s="56"/>
-      <c r="T23" s="56"/>
-      <c r="U23" s="56"/>
-      <c r="V23" s="56"/>
-      <c r="W23" s="56"/>
-      <c r="X23" s="56"/>
-      <c r="Y23" s="56"/>
-      <c r="Z23" s="56"/>
-      <c r="AA23" s="56"/>
+      <c r="A23" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="47"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="47"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="47"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="47"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="47"/>
+      <c r="M23" s="47"/>
+      <c r="N23" s="47"/>
+      <c r="O23" s="47"/>
+      <c r="P23" s="47"/>
+      <c r="Q23" s="47"/>
+      <c r="R23" s="47"/>
+      <c r="S23" s="47"/>
+      <c r="T23" s="47"/>
+      <c r="U23" s="47"/>
+      <c r="V23" s="47"/>
+      <c r="W23" s="47"/>
+      <c r="X23" s="47"/>
+      <c r="Y23" s="47"/>
+      <c r="Z23" s="47"/>
+      <c r="AA23" s="47"/>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A24" s="56"/>
-      <c r="B24" s="56"/>
-      <c r="C24" s="56"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="56"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="56"/>
-      <c r="J24" s="56"/>
-      <c r="K24" s="56"/>
-      <c r="L24" s="56"/>
-      <c r="M24" s="56"/>
-      <c r="N24" s="56"/>
-      <c r="O24" s="56"/>
-      <c r="P24" s="56"/>
-      <c r="Q24" s="56"/>
-      <c r="R24" s="56"/>
-      <c r="S24" s="56"/>
-      <c r="T24" s="56"/>
-      <c r="U24" s="56"/>
-      <c r="V24" s="56"/>
-      <c r="W24" s="56"/>
-      <c r="X24" s="56"/>
-      <c r="Y24" s="56"/>
-      <c r="Z24" s="56"/>
-      <c r="AA24" s="56"/>
+      <c r="A24" s="47"/>
+      <c r="B24" s="47"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="47"/>
+      <c r="E24" s="47"/>
+      <c r="F24" s="47"/>
+      <c r="G24" s="47"/>
+      <c r="H24" s="47"/>
+      <c r="I24" s="47"/>
+      <c r="J24" s="47"/>
+      <c r="K24" s="47"/>
+      <c r="L24" s="47"/>
+      <c r="M24" s="47"/>
+      <c r="N24" s="47"/>
+      <c r="O24" s="47"/>
+      <c r="P24" s="47"/>
+      <c r="Q24" s="47"/>
+      <c r="R24" s="47"/>
+      <c r="S24" s="47"/>
+      <c r="T24" s="47"/>
+      <c r="U24" s="47"/>
+      <c r="V24" s="47"/>
+      <c r="W24" s="47"/>
+      <c r="X24" s="47"/>
+      <c r="Y24" s="47"/>
+      <c r="Z24" s="47"/>
+      <c r="AA24" s="47"/>
     </row>
     <row r="25" spans="1:27" ht="20" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
@@ -1863,10 +1863,10 @@
         <v>11</v>
       </c>
       <c r="N25" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="O25" s="18" t="s">
         <v>27</v>
-      </c>
-      <c r="O25" s="18" t="s">
-        <v>28</v>
       </c>
       <c r="P25" s="3" t="s">
         <v>2</v>
@@ -1899,21 +1899,21 @@
         <v>11</v>
       </c>
       <c r="Z25" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA25" s="18" t="s">
         <v>27</v>
-      </c>
-      <c r="AA25" s="18" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A26" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>32</v>
       </c>
       <c r="D26" s="21"/>
       <c r="E26" s="20"/>
@@ -1944,10 +1944,10 @@
     <row r="27" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A27" s="6"/>
       <c r="B27" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="26" t="s">
         <v>46</v>
-      </c>
-      <c r="C27" s="26" t="s">
-        <v>47</v>
       </c>
       <c r="D27" s="20"/>
       <c r="E27" s="22"/>
@@ -1956,14 +1956,14 @@
       <c r="H27" s="20"/>
       <c r="I27" s="20"/>
       <c r="J27" s="20"/>
-      <c r="M27" s="48" t="s">
-        <v>13</v>
-      </c>
-      <c r="N27" s="48"/>
-      <c r="O27" s="48"/>
-      <c r="P27" s="48"/>
-      <c r="Q27" s="48"/>
-      <c r="R27" s="48"/>
+      <c r="M27" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="N27" s="56"/>
+      <c r="O27" s="56"/>
+      <c r="P27" s="56"/>
+      <c r="Q27" s="56"/>
+      <c r="R27" s="56"/>
       <c r="S27" s="20"/>
       <c r="T27" s="20"/>
       <c r="U27" s="20"/>
@@ -2002,13 +2002,13 @@
     </row>
     <row r="29" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A29" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C29" s="39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S29" s="40" t="s">
         <v>13</v>
@@ -2017,25 +2017,25 @@
     <row r="30" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A30" s="6"/>
       <c r="B30" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>72</v>
-      </c>
-      <c r="S30" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="T30" s="51"/>
+        <v>71</v>
+      </c>
+      <c r="S30" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="T30" s="59"/>
     </row>
     <row r="32" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A32" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" s="33" t="s">
         <v>54</v>
-      </c>
-      <c r="B32" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="C32" s="33" t="s">
-        <v>55</v>
       </c>
       <c r="R32" s="37"/>
       <c r="S32" s="34" t="s">
@@ -2045,10 +2045,10 @@
     <row r="33" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A33" s="30"/>
       <c r="B33" s="30" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C33" s="35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="S33" s="36" t="s">
         <v>13</v>
@@ -2057,26 +2057,26 @@
     <row r="34" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A34" s="30"/>
       <c r="B34" s="30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C34" s="38" t="s">
-        <v>56</v>
-      </c>
-      <c r="S34" s="50" t="s">
-        <v>13</v>
-      </c>
-      <c r="T34" s="50"/>
-      <c r="U34" s="50"/>
+        <v>55</v>
+      </c>
+      <c r="S34" s="58" t="s">
+        <v>13</v>
+      </c>
+      <c r="T34" s="58"/>
+      <c r="U34" s="58"/>
     </row>
     <row r="36" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A36" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="32" t="s">
         <v>65</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36" s="32" t="s">
-        <v>66</v>
       </c>
       <c r="V36" s="31" t="s">
         <v>13</v>
@@ -2085,38 +2085,38 @@
     <row r="37" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A37" s="6"/>
       <c r="B37" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="W37" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="X37" s="51"/>
+        <v>66</v>
+      </c>
+      <c r="W37" s="59" t="s">
+        <v>13</v>
+      </c>
+      <c r="X37" s="59"/>
     </row>
     <row r="38" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A38" s="6"/>
       <c r="B38" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C38" s="42" t="s">
-        <v>75</v>
-      </c>
-      <c r="W38" s="52" t="s">
-        <v>13</v>
-      </c>
-      <c r="X38" s="52"/>
+        <v>74</v>
+      </c>
+      <c r="W38" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="X38" s="60"/>
     </row>
     <row r="41" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A41" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C41" s="39" t="s">
         <v>68</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C41" s="39" t="s">
-        <v>69</v>
       </c>
       <c r="W41" s="40" t="s">
         <v>13</v>
@@ -2125,47 +2125,57 @@
     <row r="42" spans="1:27" ht="20" x14ac:dyDescent="0.15">
       <c r="A42" s="6"/>
       <c r="B42" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C42" s="27" t="s">
-        <v>70</v>
-      </c>
-      <c r="X42" s="44" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y42" s="44"/>
+        <v>69</v>
+      </c>
+      <c r="X42" s="52" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y42" s="52"/>
     </row>
     <row r="44" spans="1:27" ht="20" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C44" s="32" t="s">
-        <v>78</v>
-      </c>
-      <c r="Y44" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z44" s="45"/>
+        <v>77</v>
+      </c>
+      <c r="Y44" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z44" s="53"/>
     </row>
     <row r="45" spans="1:27" ht="20" x14ac:dyDescent="0.2">
       <c r="A45" s="6"/>
       <c r="B45" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C45" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="Y45" s="46" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z45" s="47"/>
-      <c r="AA45" s="47"/>
+        <v>78</v>
+      </c>
+      <c r="Y45" s="54" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z45" s="55"/>
+      <c r="AA45" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="X42:Y42"/>
+    <mergeCell ref="Y44:Z44"/>
+    <mergeCell ref="Y45:AA45"/>
+    <mergeCell ref="M27:R27"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="S34:U34"/>
+    <mergeCell ref="S30:T30"/>
+    <mergeCell ref="W37:X37"/>
+    <mergeCell ref="W38:X38"/>
+    <mergeCell ref="A23:AA24"/>
     <mergeCell ref="L19:M19"/>
     <mergeCell ref="P1:AA1"/>
     <mergeCell ref="D1:O1"/>
@@ -2176,16 +2186,6 @@
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="J16:K16"/>
-    <mergeCell ref="X42:Y42"/>
-    <mergeCell ref="Y44:Z44"/>
-    <mergeCell ref="Y45:AA45"/>
-    <mergeCell ref="M27:R27"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="S34:U34"/>
-    <mergeCell ref="S30:T30"/>
-    <mergeCell ref="W37:X37"/>
-    <mergeCell ref="W38:X38"/>
-    <mergeCell ref="A23:AA24"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>